<commit_message>
chore: update tiles sheet and regenerate release configs
</commit_message>
<xml_diff>
--- a/docs/design/蛋仔--大富翁--地块表.xlsx
+++ b/docs/design/蛋仔--大富翁--地块表.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\eggitor\1_开发中\大富翁\monopoly\design\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\eggitor\1_开发中\大富翁\策划案\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69F77281-ED16-49F1-8C05-F7B6937E336D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91E5FE8F-6709-445D-B49E-2FFA2D03A9FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -599,7 +599,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -624,6 +624,19 @@
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="等线"/>
       <family val="3"/>
       <charset val="134"/>
@@ -682,7 +695,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -696,6 +709,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1139,7 +1158,7 @@
         <v>1050</v>
       </c>
       <c r="H4" s="4">
-        <f t="shared" ref="G4:I4" si="2">G4*2</f>
+        <f t="shared" ref="H4:I4" si="2">G4*2</f>
         <v>2100</v>
       </c>
       <c r="I4" s="4">
@@ -1187,7 +1206,7 @@
         <v>1100</v>
       </c>
       <c r="H5" s="4">
-        <f t="shared" ref="G5:I5" si="7">G5*2</f>
+        <f t="shared" ref="H5:I5" si="7">G5*2</f>
         <v>2200</v>
       </c>
       <c r="I5" s="4">
@@ -1235,7 +1254,7 @@
         <v>1150</v>
       </c>
       <c r="H6" s="4">
-        <f t="shared" ref="G6:I6" si="8">G6*2</f>
+        <f t="shared" ref="H6:I6" si="8">G6*2</f>
         <v>2300</v>
       </c>
       <c r="I6" s="4">
@@ -1283,7 +1302,7 @@
         <v>1200</v>
       </c>
       <c r="H7" s="4">
-        <f t="shared" ref="G7:I7" si="9">G7*2</f>
+        <f t="shared" ref="H7:I7" si="9">G7*2</f>
         <v>2400</v>
       </c>
       <c r="I7" s="4">
@@ -1331,7 +1350,7 @@
         <v>1250</v>
       </c>
       <c r="H8" s="4">
-        <f t="shared" ref="G8:I8" si="10">G8*2</f>
+        <f t="shared" ref="H8:I8" si="10">G8*2</f>
         <v>2500</v>
       </c>
       <c r="I8" s="4">
@@ -1379,7 +1398,7 @@
         <v>1300</v>
       </c>
       <c r="H9" s="4">
-        <f t="shared" ref="G9:I9" si="11">G9*2</f>
+        <f t="shared" ref="H9:I9" si="11">G9*2</f>
         <v>2600</v>
       </c>
       <c r="I9" s="4">
@@ -1427,7 +1446,7 @@
         <v>1350</v>
       </c>
       <c r="H10" s="4">
-        <f t="shared" ref="G10:I10" si="12">G10*2</f>
+        <f t="shared" ref="H10:I10" si="12">G10*2</f>
         <v>2700</v>
       </c>
       <c r="I10" s="4">
@@ -1475,7 +1494,7 @@
         <v>1500</v>
       </c>
       <c r="H11" s="4">
-        <f t="shared" ref="G11:I11" si="13">G11*2</f>
+        <f t="shared" ref="H11:I11" si="13">G11*2</f>
         <v>3000</v>
       </c>
       <c r="I11" s="4">
@@ -1523,7 +1542,7 @@
         <v>1600</v>
       </c>
       <c r="H12" s="4">
-        <f t="shared" ref="G12:I12" si="14">G12*2</f>
+        <f t="shared" ref="H12:I12" si="14">G12*2</f>
         <v>3200</v>
       </c>
       <c r="I12" s="4">
@@ -1571,7 +1590,7 @@
         <v>1700</v>
       </c>
       <c r="H13" s="4">
-        <f t="shared" ref="G13:I13" si="15">G13*2</f>
+        <f t="shared" ref="H13:I13" si="15">G13*2</f>
         <v>3400</v>
       </c>
       <c r="I13" s="4">
@@ -1619,7 +1638,7 @@
         <v>1800</v>
       </c>
       <c r="H14" s="4">
-        <f t="shared" ref="G14:I14" si="16">G14*2</f>
+        <f t="shared" ref="H14:I14" si="16">G14*2</f>
         <v>3600</v>
       </c>
       <c r="I14" s="4">
@@ -1667,7 +1686,7 @@
         <v>1900</v>
       </c>
       <c r="H15" s="4">
-        <f t="shared" ref="G15:I15" si="17">G15*2</f>
+        <f t="shared" ref="H15:I15" si="17">G15*2</f>
         <v>3800</v>
       </c>
       <c r="I15" s="4">
@@ -1715,7 +1734,7 @@
         <v>2000</v>
       </c>
       <c r="H16" s="4">
-        <f t="shared" ref="G16:I16" si="18">G16*2</f>
+        <f t="shared" ref="H16:I16" si="18">G16*2</f>
         <v>4000</v>
       </c>
       <c r="I16" s="4">
@@ -1763,7 +1782,7 @@
         <v>2050</v>
       </c>
       <c r="H17" s="4">
-        <f t="shared" ref="G17:I17" si="19">G17*2</f>
+        <f t="shared" ref="H17:I17" si="19">G17*2</f>
         <v>4100</v>
       </c>
       <c r="I17" s="4">
@@ -1811,7 +1830,7 @@
         <v>2100</v>
       </c>
       <c r="H18" s="4">
-        <f t="shared" ref="G18:I18" si="20">G18*2</f>
+        <f t="shared" ref="H18:I18" si="20">G18*2</f>
         <v>4200</v>
       </c>
       <c r="I18" s="4">
@@ -1859,7 +1878,7 @@
         <v>2150</v>
       </c>
       <c r="H19" s="4">
-        <f t="shared" ref="G19:I19" si="21">G19*2</f>
+        <f t="shared" ref="H19:I19" si="21">G19*2</f>
         <v>4300</v>
       </c>
       <c r="I19" s="4">
@@ -1907,7 +1926,7 @@
         <v>2200</v>
       </c>
       <c r="H20" s="4">
-        <f t="shared" ref="G20:I20" si="22">G20*2</f>
+        <f t="shared" ref="H20:I20" si="22">G20*2</f>
         <v>4400</v>
       </c>
       <c r="I20" s="4">
@@ -1955,7 +1974,7 @@
         <v>2250</v>
       </c>
       <c r="H21" s="4">
-        <f t="shared" ref="G21:I21" si="23">G21*2</f>
+        <f t="shared" ref="H21:I21" si="23">G21*2</f>
         <v>4500</v>
       </c>
       <c r="I21" s="4">
@@ -2003,7 +2022,7 @@
         <v>2300</v>
       </c>
       <c r="H22" s="4">
-        <f t="shared" ref="G22:I22" si="24">G22*2</f>
+        <f t="shared" ref="H22:I22" si="24">G22*2</f>
         <v>4600</v>
       </c>
       <c r="I22" s="4">
@@ -2051,7 +2070,7 @@
         <v>2350</v>
       </c>
       <c r="H23" s="4">
-        <f t="shared" ref="G23:I23" si="25">G23*2</f>
+        <f t="shared" ref="H23:I23" si="25">G23*2</f>
         <v>4700</v>
       </c>
       <c r="I23" s="4">
@@ -2099,7 +2118,7 @@
         <v>2400</v>
       </c>
       <c r="H24" s="4">
-        <f t="shared" ref="G24:I24" si="26">G24*2</f>
+        <f t="shared" ref="H24:I24" si="26">G24*2</f>
         <v>4800</v>
       </c>
       <c r="I24" s="4">
@@ -2147,7 +2166,7 @@
         <v>2450</v>
       </c>
       <c r="H25" s="4">
-        <f t="shared" ref="G25:I25" si="27">G25*2</f>
+        <f t="shared" ref="H25:I25" si="27">G25*2</f>
         <v>4900</v>
       </c>
       <c r="I25" s="4">
@@ -2195,7 +2214,7 @@
         <v>2500</v>
       </c>
       <c r="H26" s="4">
-        <f t="shared" ref="G26:I26" si="28">G26*2</f>
+        <f t="shared" ref="H26:I26" si="28">G26*2</f>
         <v>5000</v>
       </c>
       <c r="I26" s="4">
@@ -2243,7 +2262,7 @@
         <v>1450</v>
       </c>
       <c r="H27" s="4">
-        <f t="shared" ref="G27:I27" si="29">G27*2</f>
+        <f t="shared" ref="H27:I27" si="29">G27*2</f>
         <v>2900</v>
       </c>
       <c r="I27" s="4">
@@ -2291,7 +2310,7 @@
         <v>1550</v>
       </c>
       <c r="H28" s="4">
-        <f t="shared" ref="G28:I28" si="30">G28*2</f>
+        <f t="shared" ref="H28:I28" si="30">G28*2</f>
         <v>3100</v>
       </c>
       <c r="I28" s="4">
@@ -2339,7 +2358,7 @@
         <v>1650</v>
       </c>
       <c r="H29" s="4">
-        <f t="shared" ref="G29:I29" si="31">G29*2</f>
+        <f t="shared" ref="H29:I29" si="31">G29*2</f>
         <v>3300</v>
       </c>
       <c r="I29" s="4">
@@ -2387,7 +2406,7 @@
         <v>1750</v>
       </c>
       <c r="H30" s="4">
-        <f t="shared" ref="G30:I30" si="32">G30*2</f>
+        <f t="shared" ref="H30:I30" si="32">G30*2</f>
         <v>3500</v>
       </c>
       <c r="I30" s="4">
@@ -2435,7 +2454,7 @@
         <v>1850</v>
       </c>
       <c r="H31" s="4">
-        <f t="shared" ref="G31:I31" si="33">G31*2</f>
+        <f t="shared" ref="H31:I31" si="33">G31*2</f>
         <v>3700</v>
       </c>
       <c r="I31" s="4">
@@ -2483,7 +2502,7 @@
         <v>1950</v>
       </c>
       <c r="H32" s="4">
-        <f t="shared" ref="G32:I32" si="34">G32*2</f>
+        <f t="shared" ref="H32:I32" si="34">G32*2</f>
         <v>3900</v>
       </c>
       <c r="I32" s="4">
@@ -2531,7 +2550,7 @@
         <v>3500</v>
       </c>
       <c r="H33" s="4">
-        <f t="shared" ref="G33:I33" si="35">G33*2</f>
+        <f t="shared" ref="H33:I33" si="35">G33*2</f>
         <v>7000</v>
       </c>
       <c r="I33" s="4">
@@ -2579,7 +2598,7 @@
         <v>4000</v>
       </c>
       <c r="H34" s="4">
-        <f t="shared" ref="G34:I34" si="36">G34*2</f>
+        <f t="shared" ref="H34:I34" si="36">G34*2</f>
         <v>8000</v>
       </c>
       <c r="I34" s="4">
@@ -2627,7 +2646,7 @@
         <v>4500</v>
       </c>
       <c r="H35" s="4">
-        <f t="shared" ref="G35:I35" si="37">G35*2</f>
+        <f t="shared" ref="H35:I35" si="37">G35*2</f>
         <v>9000</v>
       </c>
       <c r="I35" s="4">
@@ -2675,7 +2694,7 @@
         <v>5000</v>
       </c>
       <c r="H36" s="4">
-        <f t="shared" ref="G36:I36" si="38">G36*2</f>
+        <f t="shared" ref="H36:I36" si="38">G36*2</f>
         <v>10000</v>
       </c>
       <c r="I36" s="4">
@@ -2939,10 +2958,10 @@
       <c r="A42" s="1">
         <v>40</v>
       </c>
-      <c r="B42" s="6" t="s">
+      <c r="B42" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C42" s="6" t="s">
+      <c r="C42" s="8" t="s">
         <v>56</v>
       </c>
       <c r="D42" s="3" t="s">
@@ -2985,11 +3004,11 @@
       <c r="A43" s="1">
         <v>41</v>
       </c>
-      <c r="B43" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="C43" s="6" t="s">
-        <v>56</v>
+      <c r="B43" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>57</v>
       </c>
       <c r="D43" s="3" t="s">
         <v>67</v>
@@ -3031,11 +3050,11 @@
       <c r="A44" s="1">
         <v>42</v>
       </c>
-      <c r="B44" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="C44" s="6" t="s">
-        <v>56</v>
+      <c r="B44" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C44" s="7" t="s">
+        <v>57</v>
       </c>
       <c r="D44" s="3" t="s">
         <v>68</v>
@@ -3077,10 +3096,10 @@
       <c r="A45" s="1">
         <v>43</v>
       </c>
-      <c r="B45" s="6" t="s">
+      <c r="B45" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C45" s="6" t="s">
+      <c r="C45" s="8" t="s">
         <v>56</v>
       </c>
       <c r="D45" s="3" t="s">
@@ -3123,10 +3142,10 @@
       <c r="A46" s="1">
         <v>44</v>
       </c>
-      <c r="B46" s="6" t="s">
+      <c r="B46" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="C46" s="6" t="s">
+      <c r="C46" s="8" t="s">
         <v>57</v>
       </c>
       <c r="D46" s="3" t="s">
@@ -3169,11 +3188,11 @@
       <c r="A47" s="1">
         <v>45</v>
       </c>
-      <c r="B47" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="C47" s="6" t="s">
-        <v>57</v>
+      <c r="B47" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="C47" s="7" t="s">
+        <v>56</v>
       </c>
       <c r="D47" s="3" t="s">
         <v>65</v>

</xml_diff>